<commit_message>
Finished layouts and tested height calculation
</commit_message>
<xml_diff>
--- a/Раскладки.xlsx
+++ b/Раскладки.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DB\Projects\SW004-PalletWizardEco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C9F19F-4182-4497-B4A6-A4B6A1430252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD23EE0-60DB-4D4A-8F7E-E5AAD96529B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1811C202-B53B-4670-B12D-E96EADE5A5C2}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1811C202-B53B-4670-B12D-E96EADE5A5C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Раскладка 1 (5 мешков)" sheetId="1" r:id="rId1"/>
+    <sheet name="Раскладка 2 (8 мешков)" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
   <si>
     <t>Длина</t>
   </si>
@@ -75,6 +76,21 @@
   </si>
   <si>
     <t>Свисание по длинной стороне</t>
+  </si>
+  <si>
+    <t>41х37х11</t>
+  </si>
+  <si>
+    <t>49х40х11</t>
+  </si>
+  <si>
+    <t>d1max</t>
+  </si>
+  <si>
+    <t>d2</t>
+  </si>
+  <si>
+    <t>d1</t>
   </si>
 </sst>
 </file>
@@ -118,16 +134,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="25">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -140,6 +165,41 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -180,25 +240,54 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6BDA404B-FE4E-48E4-AA37-1761A6347FA2}" name="Таблица1" displayName="Таблица1" ref="A1:K5" totalsRowShown="0" headerRowDxfId="6" dataDxfId="7">
-  <autoFilter ref="A1:K5" xr:uid="{6BDA404B-FE4E-48E4-AA37-1761A6347FA2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6BDA404B-FE4E-48E4-AA37-1761A6347FA2}" name="Таблица1" displayName="Таблица1" ref="A1:K3" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:K3" xr:uid="{6BDA404B-FE4E-48E4-AA37-1761A6347FA2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C5BD9855-E1D6-49FF-B76D-93CE6D9F6868}" name="№" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{53EBF20A-6C0D-4239-A254-BA730A9D4004}" name="Типоразмер" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{AC80BA37-CDD9-4117-80FF-49507BEC419A}" name="Длина" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{49B4F7FF-F0F6-45F7-B996-2F74A72A454D}" name="Ширина" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{ABAAF6BC-A8CE-4A62-AD0D-6BC0535D2E20}" name="Свисание по короткой стороне" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{717F6A0D-44A5-409C-9975-D6DA91F79F95}" name="Свисание по длинной стороне" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{C81D9693-020B-4805-8049-483091B6F22B}" name="g1max" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{C5BD9855-E1D6-49FF-B76D-93CE6D9F6868}" name="№" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{53EBF20A-6C0D-4239-A254-BA730A9D4004}" name="Типоразмер" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{AC80BA37-CDD9-4117-80FF-49507BEC419A}" name="Длина" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{49B4F7FF-F0F6-45F7-B996-2F74A72A454D}" name="Ширина" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{ABAAF6BC-A8CE-4A62-AD0D-6BC0535D2E20}" name="Свисание по короткой стороне" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{717F6A0D-44A5-409C-9975-D6DA91F79F95}" name="Свисание по длинной стороне" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{C81D9693-020B-4805-8049-483091B6F22B}" name="g1max" dataDxfId="16">
       <calculatedColumnFormula>1000+Таблица1[[#This Row],[Свисание по короткой стороне]]*2-D2-C2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{331EC8F4-8893-47D3-A7FE-9E1A65BFB185}" name="g2max" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{331EC8F4-8893-47D3-A7FE-9E1A65BFB185}" name="g2max" dataDxfId="15">
       <calculatedColumnFormula>(1200+Таблица1[[#This Row],[Свисание по длинной стороне]]*2-3*D2)/2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0E278CC0-2AA4-4B25-8DFE-78B8FB702078}" name="g1"/>
-    <tableColumn id="6" xr3:uid="{9336F004-0A61-4313-8242-B28CD8FB31D7}" name="g2" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{CBF6D93B-3ADC-4BDE-A2CE-6E0007FD219C}" name="g3" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{9336F004-0A61-4313-8242-B28CD8FB31D7}" name="g2" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{CBF6D93B-3ADC-4BDE-A2CE-6E0007FD219C}" name="g3" dataDxfId="13">
       <calculatedColumnFormula>3*D2-2*C2+2*J2</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1172A6A4-CCEB-4F99-AF78-55560852851B}" name="Таблица13" displayName="Таблица13" ref="A1:L3" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:L3" xr:uid="{1172A6A4-CCEB-4F99-AF78-55560852851B}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{AA344718-7A34-4B2A-9BF8-6B27C125A323}" name="№" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{3B6B1069-E4C5-4E44-BDE9-2044BDE0CFE5}" name="Типоразмер" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{7C49839B-952D-4CC8-942B-D0D67FD3F709}" name="Длина" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{80F128A9-F51C-439E-9424-E16F6DB0E866}" name="Ширина" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{42E732FE-34CB-4249-9A1F-E4A87E61D395}" name="Свисание по короткой стороне" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{CD27F4A0-5218-4012-9255-FF4130DD8D29}" name="Свисание по длинной стороне" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{65BCD7B6-FFE5-4F2F-8B94-F7EDB95EF8A7}" name="g1max" dataDxfId="3">
+      <calculatedColumnFormula>(1000+Таблица13[[#This Row],[Свисание по короткой стороне]]*2-3*D2)/2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{77AE05A9-6D00-445C-98E9-6C5CCDEFE8B7}" name="d1max" dataDxfId="2">
+      <calculatedColumnFormula>(1200+Таблица13[[#This Row],[Свисание по длинной стороне]]*2-4*D2)/3</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{BEFB90B1-B127-4B31-96CA-FAD8BC6E0820}" name="g1" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{C1B249A5-B9CE-471C-AA2B-DE0E827BCF7F}" name="d1" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C661561B-BC46-4308-A62E-E96778A6DADD}" name="g2">
+      <calculatedColumnFormula>(3*Таблица13[[#This Row],[Ширина]]+3*Таблица13[[#This Row],[d1]]-2*Таблица13[[#This Row],[Длина]])/2</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{D6D34847-D3B2-438B-870F-5BAE80319891}" name="d2" dataDxfId="4">
+      <calculatedColumnFormula>3*Таблица13[[#This Row],[Ширина]]+2*Таблица13[[#This Row],[g1]]-2*Таблица13[[#This Row],[Длина]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -522,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{931A414B-31D9-481C-9AA7-0CD2213DE2D4}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -621,87 +710,41 @@
       <c r="D3" s="1">
         <v>420</v>
       </c>
-      <c r="E3" s="1">
-        <v>25</v>
+      <c r="E3" s="2">
+        <v>22.5</v>
       </c>
       <c r="F3" s="1">
         <v>35</v>
       </c>
       <c r="G3" s="1">
         <f>1000+Таблица1[[#This Row],[Свисание по короткой стороне]]*2-D3-C3</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H3" s="1">
         <f>(1200+Таблица1[[#This Row],[Свисание по длинной стороне]]*2-3*D3)/2</f>
         <v>5</v>
       </c>
       <c r="I3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J3" s="1">
         <v>5</v>
       </c>
       <c r="K3" s="1">
-        <f t="shared" ref="K3:K5" si="0">3*D3-2*C3+2*J3</f>
+        <f>3*D3-2*C3+2*J3</f>
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
+      <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="1">
-        <f>1000+Таблица1[[#This Row],[Свисание по короткой стороне]]*2-D4-C4</f>
-        <v>1000</v>
-      </c>
-      <c r="H4" s="1">
-        <f>(1200+Таблица1[[#This Row],[Свисание по длинной стороне]]*2-3*D4)/2</f>
-        <v>600</v>
-      </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1">
-        <f>1000+Таблица1[[#This Row],[Свисание по короткой стороне]]*2-D5-C5</f>
-        <v>1000</v>
-      </c>
-      <c r="H5" s="1">
-        <f>(1200+Таблица1[[#This Row],[Свисание по длинной стороне]]*2-3*D5)/2</f>
-        <v>600</v>
-      </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -710,4 +753,163 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFBC330E-366C-48B7-A662-DF7D3F348FB1}">
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="18.42578125" customWidth="1"/>
+    <col min="11" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1">
+        <v>445</v>
+      </c>
+      <c r="D2" s="1">
+        <v>305</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>20</v>
+      </c>
+      <c r="G2" s="1">
+        <f>(1000+Таблица13[[#This Row],[Свисание по короткой стороне]]*2-3*D2)/2</f>
+        <v>42.5</v>
+      </c>
+      <c r="H2" s="1">
+        <f>(1200+Таблица13[[#This Row],[Свисание по длинной стороне]]*2-4*D2)/3</f>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="I2" s="1">
+        <v>10</v>
+      </c>
+      <c r="J2" s="1">
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <f>(3*Таблица13[[#This Row],[Ширина]]+3*Таблица13[[#This Row],[d1]]-2*Таблица13[[#This Row],[Длина]])/2</f>
+        <v>20</v>
+      </c>
+      <c r="L2" s="1">
+        <f>3*Таблица13[[#This Row],[Ширина]]+2*Таблица13[[#This Row],[g1]]-2*Таблица13[[#This Row],[Длина]]</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="1">
+        <v>500</v>
+      </c>
+      <c r="D3" s="1">
+        <v>330</v>
+      </c>
+      <c r="E3" s="2">
+        <v>10</v>
+      </c>
+      <c r="F3" s="1">
+        <v>70</v>
+      </c>
+      <c r="G3" s="1">
+        <f>(1000+Таблица13[[#This Row],[Свисание по короткой стороне]]*2-3*D3)/2</f>
+        <v>15</v>
+      </c>
+      <c r="H3" s="1">
+        <f>(1200+Таблица13[[#This Row],[Свисание по длинной стороне]]*2-4*D3)/3</f>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="I3" s="1">
+        <v>10</v>
+      </c>
+      <c r="J3" s="1">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <f>(3*Таблица13[[#This Row],[Ширина]]+3*Таблица13[[#This Row],[d1]]-2*Таблица13[[#This Row],[Длина]])/2</f>
+        <v>2.5</v>
+      </c>
+      <c r="L3" s="1">
+        <f>3*Таблица13[[#This Row],[Ширина]]+2*Таблица13[[#This Row],[g1]]-2*Таблица13[[#This Row],[Длина]]</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>